<commit_message>
Battle result stats + PREP hover info + sheet-driven names
battle_screen: replace placement-cell text with unit portraits; mouse-hover panel shows unit stats + active synergies (with effects); active-synergy summary bar with effect text.

combat: CombatUnit tracks damage_dealt/kills; CombatManager aggregates MVP/total damage/kills/survivors into BattleResult; result screen shows stats for win/draw/loss.

data: fill id + display_name in Tier1_sheet (units_player, synergies_player); regenerate 24 unit + 28 synergy .tres. Units now named (e.g. 터커); synergies show 벤 보병단(N) etc. ids/filenames unchanged so references stay intact.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheet/Tier1_sheet.xlsx
+++ b/sheet/Tier1_sheet.xlsx
@@ -14,7 +14,7 @@
     <sheet name="encounters_slots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -555,6 +555,16 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ven_infantry_soldier</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>터커</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>벤</t>
@@ -617,6 +627,16 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ven_infantry_mercenary</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>크리스</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>벤</t>
@@ -679,6 +699,16 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ven_infantry_adventurer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>존</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>벤</t>
@@ -741,6 +771,16 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ven_spearman_soldier</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>해리스</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>벤</t>
@@ -803,6 +843,16 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ven_spearman_mercenary</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>케인</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>벤</t>
@@ -865,6 +915,16 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ven_spearman_adventurer</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>브렌</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>벤</t>
@@ -927,6 +987,16 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>krem_infantry_soldier</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>할리</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>크렘</t>
@@ -989,6 +1059,16 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>krem_infantry_mercenary</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>알렉스</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>크렘</t>
@@ -1051,6 +1131,16 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>krem_infantry_adventurer</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>스미스</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>크렘</t>
@@ -1113,6 +1203,16 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>krem_archer_soldier</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>에이든</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>크렘</t>
@@ -1175,6 +1275,16 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>krem_archer_mercenary</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>세르다스</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>크렘</t>
@@ -1237,6 +1347,16 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>krem_archer_adventurer</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>데미안</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>크렘</t>
@@ -1299,6 +1419,16 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>arden_archer_soldier</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>제인</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>아르덴</t>
@@ -1361,6 +1491,16 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>arden_archer_mercenary</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>메이드</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>아르덴</t>
@@ -1423,6 +1563,16 @@
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>arden_archer_adventurer</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>센크리드</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>아르덴</t>
@@ -1485,6 +1635,16 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>arden_crossbowman_mercenary</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>팜</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>아르덴</t>
@@ -1547,6 +1707,16 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>arden_crossbowman_soldier</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>트리니티</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>아르덴</t>
@@ -1609,6 +1779,16 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>arden_crossbowman_adventurer</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>레너드</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>아르덴</t>
@@ -1671,6 +1851,16 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>nelm_spearman_soldier</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>블라드</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>넬름</t>
@@ -1733,6 +1923,16 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>nelm_spearman_mercenary</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>세이지</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>넬름</t>
@@ -1795,6 +1995,16 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>nelm_spearman_adventurer</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>헤럴드</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>넬름</t>
@@ -1857,6 +2067,16 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>nelm_crossbowman_mercenary</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>르만다</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>넬름</t>
@@ -1919,6 +2139,16 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>nelm_crossbowman_soldier</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>개리</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>넬름</t>
@@ -1981,6 +2211,16 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>nelm_crossbowman_adventurer</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>운타라</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>넬름</t>
@@ -2069,7 +2309,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="3.125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="13.125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="19" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="32.5" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="14.875" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="21.75" bestFit="1" customWidth="1" min="5" max="5"/>
@@ -2078,6 +2318,14 @@
     <col width="13.5" bestFit="1" customWidth="1" min="8" max="8"/>
     <col width="23" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="16.375" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="14.625" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="17.625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="20" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="24.5" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="14.375" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="16" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="15.25" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="25.25" bestFit="1" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2173,6 +2421,16 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>syn_ven_infantry_t2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>벤 보병단(2)</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>벤 보병이 인접했을 때 발동</t>
@@ -2223,6 +2481,16 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>syn_ven_infantry_t3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>벤 보병단(3)</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>벤 보병이 인접했을 때 발동</t>
@@ -2273,6 +2541,16 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>syn_ven_infantry_t4</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>벤 보병단(4)</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>벤 보병이 인접했을 때 발동</t>
@@ -2323,6 +2601,16 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>syn_ven_infantry_t5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>벤 보병단(5)</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>벤 보병이 인접했을 때 발동</t>
@@ -2373,6 +2661,16 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>syn_ven_spearman_t2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>벤 창병단(2)</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>벤 창병이 인접했을 때 발동</t>
@@ -2423,6 +2721,16 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>syn_ven_spearman_t3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>벤 창병단(3)</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>벤 창병이 인접했을 때 발동</t>
@@ -2473,6 +2781,16 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>syn_ven_spearman_t4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>벤 창병단(4)</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>벤 창병이 인접했을 때 발동</t>
@@ -2523,6 +2841,16 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>syn_ven_spearman_t5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>벤 창병단(5)</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>벤 창병이 인접했을 때 발동</t>
@@ -2573,6 +2901,16 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>syn_arden_archer_t2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>아르덴 궁수대(2)</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>아르덴 궁병이 인접했을 때 발동</t>
@@ -2626,6 +2964,16 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>syn_arden_archer_t3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>아르덴 궁수대(3)</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>아르덴 궁병이 인접했을 때 발동</t>
@@ -2679,6 +3027,16 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>syn_arden_archer_t4</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>아르덴 궁수대(4)</t>
+        </is>
+      </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>아르덴 궁병이 인접했을 때 발동</t>
@@ -2732,6 +3090,16 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>syn_arden_crossbowman_t2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>아르덴 석궁대(2)</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>아르덴 석궁병이 인접했을 때 발동</t>
@@ -2785,6 +3153,16 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>syn_arden_crossbowman_t3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>아르덴 석궁대(3)</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>아르덴 석궁병이 인접했을 때 발동</t>
@@ -2838,6 +3216,16 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>syn_arden_crossbowman_t4</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>아르덴 석궁대(4)</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>아르덴 석궁병이 인접했을 때 발동</t>
@@ -2891,6 +3279,16 @@
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>syn_krem_infantry_t2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>크렘 철벽 보병단(2)</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>크렘 보병이 인접했을 때 발동</t>
@@ -2941,6 +3339,16 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>syn_krem_infantry_t3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>크렘 철벽 보병단(3)</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>크렘 보병이 인접했을 때 발동</t>
@@ -2991,6 +3399,16 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>syn_krem_infantry_t4</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>크렘 철벽 보병단(4)</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>크렘 보병이 인접했을 때 발동</t>
@@ -3041,6 +3459,16 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>syn_krem_infantry_t5</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>크렘 철벽 보병단(5)</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>크렘 보병이 인접했을 때 발동</t>
@@ -3091,6 +3519,16 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>syn_krem_archer_t2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>크렘 사수대(2)</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>크렘 궁병이 인접했을 때 발동</t>
@@ -3144,6 +3582,16 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>syn_krem_archer_t3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>크렘 사수대(3)</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>크렘 궁병이 인접했을 때 발동</t>
@@ -3197,6 +3645,16 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>syn_krem_archer_t4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>크렘 사수대(4)</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>크렘 궁병이 인접했을 때 발동</t>
@@ -3250,6 +3708,16 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>syn_nelm_spearman_t2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>넬름 장창 방진(2)</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>넬름 창병이 인접했을 때 발동</t>
@@ -3300,6 +3768,16 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>syn_nelm_spearman_t3</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>넬름 장창 방진(3)</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>넬름 창병이 인접했을 때 발동</t>
@@ -3350,6 +3828,16 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>syn_nelm_spearman_t4</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>넬름 장창 방진(4)</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>넬름 창병이 인접했을 때 발동</t>
@@ -3400,6 +3888,16 @@
       </c>
     </row>
     <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>syn_nelm_spearman_t5</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>넬름 장창 방진(5)</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>넬름 창병이 인접했을 때 발동</t>
@@ -3450,6 +3948,16 @@
       </c>
     </row>
     <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>syn_nelm_crossbowman_t2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>넬름 석궁대(2)</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
           <t>넬름 석궁병이 인접했을 때 발동</t>
@@ -3503,6 +4011,16 @@
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>syn_nelm_crossbowman_t3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>넬름 석궁대(3)</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>넬름 석궁병이 인접했을 때 발동</t>
@@ -3556,6 +4074,16 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>syn_nelm_crossbowman_t4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>넬름 석궁대(4)</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>넬름 석궁병이 인접했을 때 발동</t>
@@ -3622,8 +4150,8 @@
   <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
-    <col width="3.125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="13.125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="17.625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="13.75" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="8" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="6.625" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="12.625" bestFit="1" customWidth="1" min="5" max="5"/>
@@ -3632,7 +4160,15 @@
     <col width="11.75" bestFit="1" customWidth="1" min="8" max="8"/>
     <col width="7.25" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="4.25" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="6.125" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="12.75" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="8.125" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="11" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="13.375" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="17.875" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="8" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="9.375" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="8.75" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="18.625" bestFit="1" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4839,13 +5375,12 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
-    <col width="3.125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="13.125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="7.75" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="5.25" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="7.75" bestFit="1" customWidth="1" min="3" max="4"/>
     <col width="21.25" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="7.875" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="6.125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="61.75" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="35.375" bestFit="1" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>